<commit_message>
Atualização da planilha LIRAa via Painel Administrativo
</commit_message>
<xml_diff>
--- a/docs/LIRAa Dados.xlsx
+++ b/docs/LIRAa Dados.xlsx
@@ -408,7 +408,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:K68"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -435,6 +435,15 @@
       <c r="H1" t="str">
         <v>Alb</v>
       </c>
+      <c r="I1" t="str">
+        <v>Inf.Predial</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Breteau</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Alb</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -453,12 +462,21 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>-0.7</v>
+        <v>0</v>
       </c>
       <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>1.4</v>
+      </c>
+      <c r="J2">
+        <v>3.5</v>
+      </c>
+      <c r="K2">
         <v>0</v>
       </c>
     </row>
@@ -479,12 +497,21 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="G3">
         <v>0</v>
       </c>
       <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
         <v>0</v>
       </c>
     </row>
@@ -508,9 +535,18 @@
         <v>0</v>
       </c>
       <c r="G4">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
         <v>0</v>
       </c>
     </row>
@@ -531,12 +567,21 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
       <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
         <v>0</v>
       </c>
     </row>
@@ -557,12 +602,21 @@
         <v>0</v>
       </c>
       <c r="F6">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G6">
         <v>0</v>
       </c>
       <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>2.1</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
         <v>0</v>
       </c>
     </row>
@@ -583,12 +637,21 @@
         <v>0</v>
       </c>
       <c r="F7">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G7">
         <v>0</v>
       </c>
       <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
         <v>0</v>
       </c>
     </row>
@@ -609,12 +672,21 @@
         <v>0</v>
       </c>
       <c r="F8">
-        <v>-0.4</v>
+        <v>0</v>
       </c>
       <c r="G8">
         <v>0</v>
       </c>
       <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
         <v>0</v>
       </c>
     </row>
@@ -643,6 +715,15 @@
       <c r="H9">
         <v>0</v>
       </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10">
@@ -669,6 +750,15 @@
       <c r="H10">
         <v>0</v>
       </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11">
@@ -687,12 +777,21 @@
         <v>0</v>
       </c>
       <c r="F11">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="G11">
         <v>0</v>
       </c>
       <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
         <v>0</v>
       </c>
     </row>
@@ -721,6 +820,15 @@
       <c r="H12">
         <v>0</v>
       </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -747,6 +855,15 @@
       <c r="H13">
         <v>0</v>
       </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -773,6 +890,15 @@
       <c r="H14">
         <v>0</v>
       </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15">
@@ -799,6 +925,15 @@
       <c r="H15">
         <v>0</v>
       </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16">
@@ -820,10 +955,19 @@
         <v>0</v>
       </c>
       <c r="G16">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="H16">
-        <v>2.7</v>
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -851,6 +995,15 @@
       <c r="H17">
         <v>0</v>
       </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18">
@@ -877,6 +1030,15 @@
       <c r="H18">
         <v>0</v>
       </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19">
@@ -903,6 +1065,15 @@
       <c r="H19">
         <v>0</v>
       </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20">
@@ -929,6 +1100,15 @@
       <c r="H20">
         <v>0</v>
       </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21">
@@ -955,6 +1135,15 @@
       <c r="H21">
         <v>0</v>
       </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="K21">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22">
@@ -981,6 +1170,15 @@
       <c r="H22">
         <v>0</v>
       </c>
+      <c r="I22">
+        <v>0</v>
+      </c>
+      <c r="J22">
+        <v>0</v>
+      </c>
+      <c r="K22">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23">
@@ -999,12 +1197,21 @@
         <v>0</v>
       </c>
       <c r="F23">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="G23">
         <v>0</v>
       </c>
       <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
         <v>0</v>
       </c>
     </row>
@@ -1033,6 +1240,15 @@
       <c r="H24">
         <v>0</v>
       </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25">
@@ -1059,6 +1275,15 @@
       <c r="H25">
         <v>0</v>
       </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26">
@@ -1085,6 +1310,15 @@
       <c r="H26">
         <v>0</v>
       </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27">
@@ -1111,6 +1345,15 @@
       <c r="H27">
         <v>0</v>
       </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28">
@@ -1137,6 +1380,15 @@
       <c r="H28">
         <v>0</v>
       </c>
+      <c r="I28">
+        <v>0</v>
+      </c>
+      <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29">
@@ -1163,6 +1415,15 @@
       <c r="H29">
         <v>0</v>
       </c>
+      <c r="I29">
+        <v>0</v>
+      </c>
+      <c r="J29">
+        <v>0</v>
+      </c>
+      <c r="K29">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30">
@@ -1189,6 +1450,15 @@
       <c r="H30">
         <v>0</v>
       </c>
+      <c r="I30">
+        <v>0</v>
+      </c>
+      <c r="J30">
+        <v>0</v>
+      </c>
+      <c r="K30">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31">
@@ -1215,6 +1485,15 @@
       <c r="H31">
         <v>0</v>
       </c>
+      <c r="I31">
+        <v>0</v>
+      </c>
+      <c r="J31">
+        <v>0</v>
+      </c>
+      <c r="K31">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32">
@@ -1241,6 +1520,15 @@
       <c r="H32">
         <v>0</v>
       </c>
+      <c r="I32">
+        <v>0</v>
+      </c>
+      <c r="J32">
+        <v>0</v>
+      </c>
+      <c r="K32">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33">
@@ -1267,6 +1555,15 @@
       <c r="H33">
         <v>0</v>
       </c>
+      <c r="I33">
+        <v>0</v>
+      </c>
+      <c r="J33">
+        <v>0</v>
+      </c>
+      <c r="K33">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34">
@@ -1293,6 +1590,15 @@
       <c r="H34">
         <v>0</v>
       </c>
+      <c r="I34">
+        <v>0</v>
+      </c>
+      <c r="J34">
+        <v>0</v>
+      </c>
+      <c r="K34">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35">
@@ -1319,6 +1625,15 @@
       <c r="H35">
         <v>0</v>
       </c>
+      <c r="I35">
+        <v>0</v>
+      </c>
+      <c r="J35">
+        <v>0</v>
+      </c>
+      <c r="K35">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36">
@@ -1345,6 +1660,15 @@
       <c r="H36">
         <v>0</v>
       </c>
+      <c r="I36">
+        <v>0</v>
+      </c>
+      <c r="J36">
+        <v>0</v>
+      </c>
+      <c r="K36">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37">
@@ -1371,6 +1695,15 @@
       <c r="H37">
         <v>0</v>
       </c>
+      <c r="I37">
+        <v>0</v>
+      </c>
+      <c r="J37">
+        <v>0</v>
+      </c>
+      <c r="K37">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38">
@@ -1397,6 +1730,15 @@
       <c r="H38">
         <v>0</v>
       </c>
+      <c r="I38">
+        <v>0</v>
+      </c>
+      <c r="J38">
+        <v>0</v>
+      </c>
+      <c r="K38">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39">
@@ -1423,6 +1765,15 @@
       <c r="H39">
         <v>0</v>
       </c>
+      <c r="I39">
+        <v>0</v>
+      </c>
+      <c r="J39">
+        <v>0</v>
+      </c>
+      <c r="K39">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40">
@@ -1449,6 +1800,15 @@
       <c r="H40">
         <v>0</v>
       </c>
+      <c r="I40">
+        <v>0</v>
+      </c>
+      <c r="J40">
+        <v>0</v>
+      </c>
+      <c r="K40">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41">
@@ -1475,6 +1835,15 @@
       <c r="H41">
         <v>0</v>
       </c>
+      <c r="I41">
+        <v>0</v>
+      </c>
+      <c r="J41">
+        <v>0</v>
+      </c>
+      <c r="K41">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42">
@@ -1501,6 +1870,15 @@
       <c r="H42">
         <v>0</v>
       </c>
+      <c r="I42">
+        <v>0</v>
+      </c>
+      <c r="J42">
+        <v>0</v>
+      </c>
+      <c r="K42">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43">
@@ -1527,6 +1905,15 @@
       <c r="H43">
         <v>0</v>
       </c>
+      <c r="I43">
+        <v>0</v>
+      </c>
+      <c r="J43">
+        <v>0</v>
+      </c>
+      <c r="K43">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44">
@@ -1553,6 +1940,15 @@
       <c r="H44">
         <v>0</v>
       </c>
+      <c r="I44">
+        <v>0</v>
+      </c>
+      <c r="J44">
+        <v>0</v>
+      </c>
+      <c r="K44">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45">
@@ -1579,6 +1975,15 @@
       <c r="H45">
         <v>0</v>
       </c>
+      <c r="I45">
+        <v>0</v>
+      </c>
+      <c r="J45">
+        <v>0</v>
+      </c>
+      <c r="K45">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46">
@@ -1605,6 +2010,15 @@
       <c r="H46">
         <v>0</v>
       </c>
+      <c r="I46">
+        <v>0</v>
+      </c>
+      <c r="J46">
+        <v>0</v>
+      </c>
+      <c r="K46">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47">
@@ -1631,6 +2045,15 @@
       <c r="H47">
         <v>0</v>
       </c>
+      <c r="I47">
+        <v>0</v>
+      </c>
+      <c r="J47">
+        <v>0</v>
+      </c>
+      <c r="K47">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48">
@@ -1657,6 +2080,15 @@
       <c r="H48">
         <v>0</v>
       </c>
+      <c r="I48">
+        <v>0</v>
+      </c>
+      <c r="J48">
+        <v>0</v>
+      </c>
+      <c r="K48">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49">
@@ -1683,6 +2115,15 @@
       <c r="H49">
         <v>0</v>
       </c>
+      <c r="I49">
+        <v>0</v>
+      </c>
+      <c r="J49">
+        <v>0</v>
+      </c>
+      <c r="K49">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50">
@@ -1709,6 +2150,15 @@
       <c r="H50">
         <v>0</v>
       </c>
+      <c r="I50">
+        <v>0</v>
+      </c>
+      <c r="J50">
+        <v>0</v>
+      </c>
+      <c r="K50">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51">
@@ -1735,6 +2185,15 @@
       <c r="H51">
         <v>0</v>
       </c>
+      <c r="I51">
+        <v>0</v>
+      </c>
+      <c r="J51">
+        <v>0</v>
+      </c>
+      <c r="K51">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52">
@@ -1761,6 +2220,15 @@
       <c r="H52">
         <v>0</v>
       </c>
+      <c r="I52">
+        <v>0</v>
+      </c>
+      <c r="J52">
+        <v>0</v>
+      </c>
+      <c r="K52">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53">
@@ -1787,6 +2255,15 @@
       <c r="H53">
         <v>0</v>
       </c>
+      <c r="I53">
+        <v>0</v>
+      </c>
+      <c r="J53">
+        <v>0</v>
+      </c>
+      <c r="K53">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54">
@@ -1813,6 +2290,15 @@
       <c r="H54">
         <v>0</v>
       </c>
+      <c r="I54">
+        <v>0</v>
+      </c>
+      <c r="J54">
+        <v>0</v>
+      </c>
+      <c r="K54">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55">
@@ -1839,6 +2325,15 @@
       <c r="H55">
         <v>0</v>
       </c>
+      <c r="I55">
+        <v>0</v>
+      </c>
+      <c r="J55">
+        <v>0</v>
+      </c>
+      <c r="K55">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56">
@@ -1865,6 +2360,15 @@
       <c r="H56">
         <v>0</v>
       </c>
+      <c r="I56">
+        <v>0</v>
+      </c>
+      <c r="J56">
+        <v>0</v>
+      </c>
+      <c r="K56">
+        <v>0</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57">
@@ -1891,6 +2395,15 @@
       <c r="H57">
         <v>0</v>
       </c>
+      <c r="I57">
+        <v>0</v>
+      </c>
+      <c r="J57">
+        <v>0</v>
+      </c>
+      <c r="K57">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58">
@@ -1917,6 +2430,15 @@
       <c r="H58">
         <v>0</v>
       </c>
+      <c r="I58">
+        <v>0</v>
+      </c>
+      <c r="J58">
+        <v>0</v>
+      </c>
+      <c r="K58">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59">
@@ -1943,6 +2465,15 @@
       <c r="H59">
         <v>0</v>
       </c>
+      <c r="I59">
+        <v>0</v>
+      </c>
+      <c r="J59">
+        <v>0</v>
+      </c>
+      <c r="K59">
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60">
@@ -1969,6 +2500,15 @@
       <c r="H60">
         <v>0</v>
       </c>
+      <c r="I60">
+        <v>0</v>
+      </c>
+      <c r="J60">
+        <v>0</v>
+      </c>
+      <c r="K60">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61">
@@ -1995,6 +2535,15 @@
       <c r="H61">
         <v>0</v>
       </c>
+      <c r="I61">
+        <v>0</v>
+      </c>
+      <c r="J61">
+        <v>0</v>
+      </c>
+      <c r="K61">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62">
@@ -2021,6 +2570,15 @@
       <c r="H62">
         <v>0</v>
       </c>
+      <c r="I62">
+        <v>0</v>
+      </c>
+      <c r="J62">
+        <v>0</v>
+      </c>
+      <c r="K62">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63">
@@ -2047,6 +2605,15 @@
       <c r="H63">
         <v>0</v>
       </c>
+      <c r="I63">
+        <v>0</v>
+      </c>
+      <c r="J63">
+        <v>0</v>
+      </c>
+      <c r="K63">
+        <v>0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64">
@@ -2073,6 +2640,15 @@
       <c r="H64">
         <v>0</v>
       </c>
+      <c r="I64">
+        <v>0</v>
+      </c>
+      <c r="J64">
+        <v>0</v>
+      </c>
+      <c r="K64">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -2091,13 +2667,22 @@
         <v>0.0</v>
       </c>
       <c r="F65" t="str">
-        <v>0.5</v>
+        <v>0.0</v>
       </c>
       <c r="G65" t="str">
         <v>0.0</v>
       </c>
       <c r="H65" t="str">
-        <v>2.7</v>
+        <v>0.0</v>
+      </c>
+      <c r="I65" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="J65" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="K65" t="str">
+        <v>0.0</v>
       </c>
     </row>
     <row r="66">
@@ -2116,15 +2701,26 @@
         <v>C2</v>
       </c>
       <c r="B67" t="str">
-        <v>01/09/2026</v>
+        <v>12/12/2026</v>
       </c>
       <c r="C67" t="str">
-        <v>25/09/2026</v>
+        <v>20/12/2026</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>C3</v>
+      </c>
+      <c r="B68" t="str">
+        <v>02/09/2026</v>
+      </c>
+      <c r="C68" t="str">
+        <v>04/09/2026</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H67"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K68"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>